<commit_message>
feat: combine relevant sheet in the flagged cases
</commit_message>
<xml_diff>
--- a/notebooks/excluded-flagged-cases.xlsx
+++ b/notebooks/excluded-flagged-cases.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D117"/>
+  <dimension ref="A1:D122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2103,139 +2103,139 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>[2023] HKDC 1247</t>
+          <t>[2023] HKDC 720</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>user.8</t>
+          <t>user.17</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>User 8 - Zou Jincheng, Zoey</t>
+          <t>User 17 - He Fangyi, Joanna</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>zoeyischeng@connect.hku.hk</t>
+          <t>hphiii3355@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>[2023] HKCFI 654</t>
+          <t>[2023] HKDC 1247</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>user.15</t>
+          <t>user.8</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>User 15 - Leung Hoi Ching, Julie</t>
+          <t>User 8 - Zou Jincheng, Zoey</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>julie223@connect.hku.hk</t>
+          <t>zoeyischeng@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>[2024] HKCFI 2758</t>
+          <t>[2023] HKCFI 654</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>user.39</t>
+          <t>user.15</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>User 39 - Lai Yan Kiu, Ivana</t>
+          <t>User 15 - Leung Hoi Ching, Julie</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>u3640281@connect.hku.hk</t>
+          <t>julie223@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>[2024] HKCFI 2724</t>
+          <t>[2024] HKCFI 2758</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>user.21</t>
+          <t>user.39</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>User 21 - CHOI Hoi Yeung, Shannon</t>
+          <t>User 39 - Lai Yan Kiu, Ivana</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>chys@connect.hku.hk</t>
+          <t>u3640281@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>[2023] HKDC 157</t>
+          <t>[2024] HKCFI 2724</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>user.15</t>
+          <t>user.21</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>User 15 - Leung Hoi Ching, Julie</t>
+          <t>User 21 - CHOI Hoi Yeung, Shannon</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>julie223@connect.hku.hk</t>
+          <t>chys@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>[2024] HKCFI 3375</t>
+          <t>[2023] HKDC 157</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>user.21</t>
+          <t>user.15</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>User 21 - CHOI Hoi Yeung, Shannon</t>
+          <t>User 15 - Leung Hoi Ching, Julie</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>chys@connect.hku.hk</t>
+          <t>julie223@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>[2024] HKDC 1060</t>
+          <t>[2024] HKCFI 3375</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2257,29 +2257,29 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>[2024] HKCFI 3119</t>
+          <t>[2024] HKDC 1060</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>user.4</t>
+          <t>user.21</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>User 4 - Chloe Chow</t>
+          <t>User 21 - CHOI Hoi Yeung, Shannon</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>chloe1@connect.hku.hk</t>
+          <t>chys@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>[2024] HKCFI 2956</t>
+          <t>[2024] HKCFI 3119</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2301,139 +2301,139 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>[2023] HKCFI 3371</t>
+          <t>[2024] HKCFI 2956</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>user.40</t>
+          <t>user.4</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>User 40 - Ng Pui Tak, Matthew</t>
+          <t>User 4 - Chloe Chow</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>u3607618@connect.hku.hk</t>
+          <t>chloe1@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>[2023] HKCFI 1614</t>
+          <t>[2023] HKCFI 3371</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>user.1</t>
+          <t>user.40</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>User 1 - Brenda Fung</t>
+          <t>User 40 - Ng Pui Tak, Matthew</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>brendafung@connect.hku.hk</t>
+          <t>u3607618@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>[2025] HKCFI 1003</t>
+          <t>[2023] HKCFI 1614</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>user.38</t>
+          <t>user.1</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>User 38 - Wong Tsz Yan, Alyssa</t>
+          <t>User 1 - Brenda Fung</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>alyssaty@connect.hku.hk</t>
+          <t>brendafung@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>[2022] HKDC 1293</t>
+          <t>[2025] HKCFI 1003</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>user.6</t>
+          <t>user.38</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>User 6 - Sung Yan Ling</t>
+          <t>User 38 - Wong Tsz Yan, Alyssa</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>u3640306@connect.hku.hk</t>
+          <t>alyssaty@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>[2024] HKCFI 1908</t>
+          <t>[2022] HKDC 1293</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>user.4</t>
+          <t>user.6</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>User 4 - Chloe Chow</t>
+          <t>User 6 - Sung Yan Ling</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>chloe1@connect.hku.hk</t>
+          <t>u3640306@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>[2024] HKCFI 2967</t>
+          <t>[2024] HKCFI 1908</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>user.10</t>
+          <t>user.4</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>User 10 - Ma Yin Ka, Otto</t>
+          <t>User 4 - Chloe Chow</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>ottomyk@connect.hku.hk</t>
+          <t>chloe1@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>[2024] HKDC 477</t>
+          <t>[2024] HKCFI 2967</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2455,29 +2455,29 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>[2025] HKCFI 2559</t>
+          <t>[2024] HKDC 477</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>user.4</t>
+          <t>user.10</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>User 4 - Chloe Chow</t>
+          <t>User 10 - Ma Yin Ka, Otto</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>chloe1@connect.hku.hk</t>
+          <t>ottomyk@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>[2025] HKDC 2152</t>
+          <t>[2025] HKCFI 2559</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2499,161 +2499,161 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>[2023] HKDC 1167</t>
+          <t>[2025] HKDC 2152</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>user.10</t>
+          <t>user.4</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>User 10 - Ma Yin Ka, Otto</t>
+          <t>User 4 - Chloe Chow</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>ottomyk@connect.hku.hk</t>
+          <t>chloe1@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>[2023] HKCFI 1482</t>
+          <t>[2023] HKDC 1167</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>user.20</t>
+          <t>user.10</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>User 20 - Cheung Ka-Lun, Karen</t>
+          <t>User 10 - Ma Yin Ka, Otto</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>karen.c13@connect.hku.hk</t>
+          <t>ottomyk@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>[2023] HKDC 1843</t>
+          <t>[2023] HKCFI 1482</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>user.21</t>
+          <t>user.20</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>User 21 - CHOI Hoi Yeung, Shannon</t>
+          <t>User 20 - Cheung Ka-Lun, Karen</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>chys@connect.hku.hk</t>
+          <t>karen.c13@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>[2021] HKCFI 3031</t>
+          <t>[2023] HKDC 1843</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>user.5</t>
+          <t>user.21</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>User 5 - Chan Yuet Chi, Jasmine</t>
+          <t>User 21 - CHOI Hoi Yeung, Shannon</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>u3633374@connect.hku.hk</t>
+          <t>chys@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>[2024] HKCFI 3639</t>
+          <t>[2021] HKCFI 3031</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>user.3</t>
+          <t>user.5</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>User 3 - Wong Man Hei, Pheobe</t>
+          <t>User 5 - Chan Yuet Chi, Jasmine</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>wongmanheipheobe@connect.hku.hk</t>
+          <t>u3633374@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>[2022] HKCFI 3370</t>
+          <t>[2024] HKCFI 3639</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>user.15</t>
+          <t>user.3</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>User 15 - Leung Hoi Ching, Julie</t>
+          <t>User 3 - Wong Man Hei, Pheobe</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>julie223@connect.hku.hk</t>
+          <t>wongmanheipheobe@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>[2025] HKCFI 5547</t>
+          <t>[2022] HKCFI 3370</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>user.34</t>
+          <t>user.15</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>User 34 - Zhang Yuen Ka, Winnie</t>
+          <t>User 15 - Leung Hoi Ching, Julie</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>winniezyk@connect.hku.hk</t>
+          <t>julie223@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>[2025] HKCFI 699</t>
+          <t>[2025] HKCFI 5547</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2675,95 +2675,95 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>[2022] HKDC 587</t>
+          <t>[2025] HKCFI 699</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>user.6</t>
+          <t>user.34</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>User 6 - Sung Yan Ling</t>
+          <t>User 34 - Zhang Yuen Ka, Winnie</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>u3640306@connect.hku.hk</t>
+          <t>winniezyk@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>[2025] HKCFI 993</t>
+          <t>[2024] HKDC 1792</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>user.3</t>
+          <t>user.2</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>User 3 - Wong Man Hei, Pheobe</t>
+          <t>User 2 - Wong Hoi Tung, Zoe</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>wongmanheipheobe@connect.hku.hk</t>
+          <t>u3640187@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>[2022] HKDC 198</t>
+          <t>[2022] HKDC 1458</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>user.3</t>
+          <t>user.9</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>User 3 - Wong Man Hei, Pheobe</t>
+          <t>User 9 - Xu Wenxuan</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>wongmanheipheobe@connect.hku.hk</t>
+          <t>jonwardxu@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>[2022] HKDC 1522</t>
+          <t>[2022] HKDC 587</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>user.3</t>
+          <t>user.6</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>User 3 - Wong Man Hei, Pheobe</t>
+          <t>User 6 - Sung Yan Ling</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>wongmanheipheobe@connect.hku.hk</t>
+          <t>u3640306@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>[2022] HKDC 1469</t>
+          <t>[2025] HKCFI 993</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2785,220 +2785,330 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>[2023] HKCFI 1074</t>
+          <t>[2022] HKDC 198</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>user.38</t>
+          <t>user.3</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>User 38 - Wong Tsz Yan, Alyssa</t>
+          <t>User 3 - Wong Man Hei, Pheobe</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>alyssaty@connect.hku.hk</t>
+          <t>wongmanheipheobe@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>[2023] HKDC 1399</t>
+          <t>[2022] HKDC 1522</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>user.37</t>
+          <t>user.3</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>User 37 - Lam Pui Man, Linda</t>
+          <t>User 3 - Wong Man Hei, Pheobe</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>linda235@connect.hku.hk</t>
+          <t>wongmanheipheobe@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>[2022] HKDC 1150</t>
+          <t>[2024] HKDC 589</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>user.15</t>
+          <t>user.2</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>User 15 - Leung Hoi Ching, Julie</t>
+          <t>User 2 - Wong Hoi Tung, Zoe</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>julie223@connect.hku.hk</t>
+          <t>u3640187@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>[2022] HKDC 1319</t>
+          <t>[2022] HKDC 1469</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>user.15</t>
+          <t>user.3</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>User 15 - Leung Hoi Ching, Julie</t>
+          <t>User 3 - Wong Man Hei, Pheobe</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>julie223@connect.hku.hk</t>
+          <t>wongmanheipheobe@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>[2024] HKDC 1239</t>
+          <t>[2023] HKCFI 1074</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>user.32</t>
+          <t>user.38</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>User 32 - Kulpriya Lam</t>
+          <t>User 38 - Wong Tsz Yan, Alyssa</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>kulpriya@connect.hku.hk</t>
+          <t>alyssaty@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>[2021] HKCFI 2663</t>
+          <t>[2023] HKDC 1399</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>user.12</t>
+          <t>user.37</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>User 12 - WU Yangyi</t>
+          <t>User 37 - Lam Pui Man, Linda</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>u3597419@connect.hku.hk</t>
+          <t>linda235@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>[2021] HKCFI 3788</t>
+          <t>[2022] HKDC 1150</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>user.12</t>
+          <t>user.15</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>User 12 - WU Yangyi</t>
+          <t>User 15 - Leung Hoi Ching, Julie</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>u3597419@connect.hku.hk</t>
+          <t>julie223@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>[2022] HKDC 146</t>
+          <t>[2022] HKDC 1319</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>user.10</t>
+          <t>user.15</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>User 10 - Ma Yin Ka, Otto</t>
+          <t>User 15 - Leung Hoi Ching, Julie</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>ottomyk@connect.hku.hk</t>
+          <t>julie223@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>[2021] HKDC 1170</t>
+          <t>[2024] HKDC 1239</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>user.10</t>
+          <t>user.32</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>User 10 - Ma Yin Ka, Otto</t>
+          <t>User 32 - Kulpriya Lam</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>ottomyk@connect.hku.hk</t>
+          <t>kulpriya@connect.hku.hk</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
+          <t>[2021] HKCFI 2663</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>user.12</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>User 12 - WU Yangyi</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>u3597419@connect.hku.hk</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>[2021] HKCFI 3788</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>user.12</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>User 12 - WU Yangyi</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>u3597419@connect.hku.hk</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>[2022] HKDC 146</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>user.10</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>User 10 - Ma Yin Ka, Otto</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>ottomyk@connect.hku.hk</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>[2021] HKDC 1170</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>user.10</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>User 10 - Ma Yin Ka, Otto</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>ottomyk@connect.hku.hk</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
           <t>[2025] HKCFI 3531</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B121" t="inlineStr">
         <is>
           <t>super.admin</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>Super Admin</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr">
+      <c r="D121" t="inlineStr">
         <is>
           <t>admin@admin.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>[2024] HKCFI 3332</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>user.20</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>User 20 - Cheung Ka-Lun, Karen</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>karen.c13@connect.hku.hk</t>
         </is>
       </c>
     </row>

</xml_diff>